<commit_message>
created .bat and momentum folder
</commit_message>
<xml_diff>
--- a/final_result/momentum_us_etfs_ranked.xlsx
+++ b/final_result/momentum_us_etfs_ranked.xlsx
@@ -471,32 +471,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>EWY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9</v>
+        <v>4.4</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>37.1</v>
+        <v>29.9</v>
       </c>
       <c r="E2" t="n">
-        <v>34.6</v>
+        <v>35.3</v>
       </c>
       <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
         <v>3</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -505,32 +505,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EWT</t>
+          <t>DXYZ</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.1</v>
+        <v>29</v>
       </c>
       <c r="C3" t="n">
-        <v>8.1</v>
+        <v>31.6</v>
       </c>
       <c r="D3" t="n">
-        <v>27.1</v>
+        <v>37.2</v>
       </c>
       <c r="E3" t="n">
-        <v>32.2</v>
+        <v>24.9</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
         <v>3</v>
-      </c>
-      <c r="H3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.8</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
@@ -539,32 +539,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EWY</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.8</v>
+        <v>1.5</v>
       </c>
       <c r="C4" t="n">
-        <v>6.3</v>
+        <v>10.7</v>
       </c>
       <c r="D4" t="n">
-        <v>31.8</v>
+        <v>34.3</v>
       </c>
       <c r="E4" t="n">
-        <v>32.3</v>
+        <v>31.1</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -573,32 +573,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ICLN</t>
+          <t>EWT</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>16.1</v>
+        <v>26.8</v>
       </c>
       <c r="E5" t="n">
-        <v>15.4</v>
+        <v>31.1</v>
       </c>
       <c r="F5" t="n">
         <v>6</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="I5" t="n">
-        <v>6.4</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="J5" t="n">
         <v>4</v>
@@ -607,32 +607,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>ICLN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2.9</v>
       </c>
       <c r="C6" t="n">
-        <v>4.9</v>
+        <v>5.6</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>12.6</v>
+        <v>13.9</v>
       </c>
       <c r="F6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H6" t="n">
         <v>9</v>
       </c>
       <c r="I6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.200000000000001</v>
       </c>
       <c r="J6" t="n">
         <v>5</v>
@@ -641,32 +641,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MTUM</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="C7" t="n">
-        <v>3.9</v>
+        <v>4.8</v>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>18.5</v>
       </c>
       <c r="E7" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="F7" t="n">
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
       <c r="G7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I7" t="n">
-        <v>10.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J7" t="n">
         <v>6</v>
@@ -675,32 +675,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.5</v>
+        <v>9.6</v>
       </c>
       <c r="C8" t="n">
-        <v>3.9</v>
+        <v>21.7</v>
       </c>
       <c r="D8" t="n">
-        <v>15.2</v>
+        <v>6.2</v>
       </c>
       <c r="E8" t="n">
-        <v>8.5</v>
+        <v>96</v>
       </c>
       <c r="F8" t="n">
-        <v>15.5</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>8</v>
+        <v>20.5</v>
       </c>
       <c r="H8" t="n">
-        <v>14.5</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>12.1</v>
+        <v>9.000000000000002</v>
       </c>
       <c r="J8" t="n">
         <v>7</v>
@@ -709,32 +709,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TAN</t>
+          <t>DBC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.6</v>
+        <v>4.1</v>
       </c>
       <c r="C9" t="n">
-        <v>7.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>8.1</v>
+        <v>6.3</v>
       </c>
       <c r="E9" t="n">
-        <v>10.1</v>
+        <v>33.1</v>
       </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H9" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
-        <v>13.4</v>
+        <v>9.600000000000001</v>
       </c>
       <c r="J9" t="n">
         <v>8</v>
@@ -743,32 +743,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EEM</t>
+          <t>MTUM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8</v>
+        <v>3.9</v>
       </c>
       <c r="D10" t="n">
-        <v>13.3</v>
+        <v>14.8</v>
       </c>
       <c r="E10" t="n">
-        <v>8.5</v>
+        <v>10.1</v>
       </c>
       <c r="F10" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G10" t="n">
-        <v>10.5</v>
+        <v>7</v>
       </c>
       <c r="H10" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="I10" t="n">
-        <v>14.4</v>
+        <v>11.6</v>
       </c>
       <c r="J10" t="n">
         <v>9</v>
@@ -777,32 +777,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DBC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.2</v>
+        <v>1.3</v>
       </c>
       <c r="C11" t="n">
-        <v>8.9</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>14.3</v>
       </c>
       <c r="E11" t="n">
-        <v>26.1</v>
+        <v>7.6</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G11" t="n">
-        <v>30.5</v>
+        <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="I11" t="n">
-        <v>15</v>
+        <v>13.8</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>

</xml_diff>